<commit_message>
Add PDF download feature and update notification data
- Added PDF download buttons for all reports (CSV + PDF options)
- Added reportlab library for PDF generation
- Updated data_service.py with CSV validation
- Fixed bottom_25 variable naming consistency
- Updated notification data (115,853 records)
- Added convert_summary_to_pdf.py script
- Updated requirements.txt with reportlab and pillow
</commit_message>
<xml_diff>
--- a/Eco-Club-Complete_Summary.xlsx
+++ b/Eco-Club-Complete_Summary.xlsx
@@ -463,10 +463,10 @@
         <v>1077</v>
       </c>
       <c r="C2" t="n">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="D2" t="n">
-        <v>24.33</v>
+        <v>26.74</v>
       </c>
     </row>
     <row r="3">
@@ -495,10 +495,10 @@
         <v>429</v>
       </c>
       <c r="C4" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D4" t="n">
-        <v>71.79000000000001</v>
+        <v>72.03</v>
       </c>
     </row>
     <row r="5">
@@ -511,10 +511,10 @@
         <v>274</v>
       </c>
       <c r="C5" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D5" t="n">
-        <v>52.19</v>
+        <v>52.55</v>
       </c>
     </row>
     <row r="6">
@@ -543,10 +543,10 @@
         <v>838</v>
       </c>
       <c r="C7" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D7" t="n">
-        <v>19.57</v>
+        <v>20.17</v>
       </c>
     </row>
     <row r="8">
@@ -559,10 +559,10 @@
         <v>218</v>
       </c>
       <c r="C8" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D8" t="n">
-        <v>41.74</v>
+        <v>42.66</v>
       </c>
     </row>
     <row r="9">
@@ -575,10 +575,10 @@
         <v>330</v>
       </c>
       <c r="C9" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D9" t="n">
-        <v>30.91</v>
+        <v>31.21</v>
       </c>
     </row>
     <row r="10">
@@ -591,10 +591,10 @@
         <v>625</v>
       </c>
       <c r="C10" t="n">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="D10" t="n">
-        <v>36.32</v>
+        <v>37.28</v>
       </c>
     </row>
     <row r="11">
@@ -639,10 +639,10 @@
         <v>354</v>
       </c>
       <c r="C13" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D13" t="n">
-        <v>42.66</v>
+        <v>42.94</v>
       </c>
     </row>
     <row r="14">
@@ -655,10 +655,10 @@
         <v>529</v>
       </c>
       <c r="C14" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D14" t="n">
-        <v>51.23</v>
+        <v>51.42</v>
       </c>
     </row>
     <row r="15">
@@ -671,10 +671,10 @@
         <v>442</v>
       </c>
       <c r="C15" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D15" t="n">
-        <v>40.27</v>
+        <v>40.72</v>
       </c>
     </row>
     <row r="16">
@@ -687,10 +687,10 @@
         <v>231</v>
       </c>
       <c r="C16" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D16" t="n">
-        <v>61.04</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="17">
@@ -703,10 +703,10 @@
         <v>528</v>
       </c>
       <c r="C17" t="n">
-        <v>241</v>
+        <v>290</v>
       </c>
       <c r="D17" t="n">
-        <v>45.64</v>
+        <v>54.92</v>
       </c>
     </row>
     <row r="18">
@@ -719,10 +719,10 @@
         <v>324</v>
       </c>
       <c r="C18" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D18" t="n">
-        <v>33.64</v>
+        <v>34.26</v>
       </c>
     </row>
     <row r="19">
@@ -767,10 +767,10 @@
         <v>134</v>
       </c>
       <c r="C21" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D21" t="n">
-        <v>63.43</v>
+        <v>64.18000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -831,10 +831,10 @@
         <v>525</v>
       </c>
       <c r="C25" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D25" t="n">
-        <v>47.05</v>
+        <v>47.24</v>
       </c>
     </row>
     <row r="26">
@@ -863,10 +863,10 @@
         <v>463</v>
       </c>
       <c r="C27" t="n">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="D27" t="n">
-        <v>55.72</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="28">
@@ -911,10 +911,10 @@
         <v>455</v>
       </c>
       <c r="C30" t="n">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D30" t="n">
-        <v>54.73</v>
+        <v>54.95</v>
       </c>
     </row>
     <row r="31">
@@ -927,10 +927,10 @@
         <v>949</v>
       </c>
       <c r="C31" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="D31" t="n">
-        <v>9.59</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="32">
@@ -943,10 +943,10 @@
         <v>540</v>
       </c>
       <c r="C32" t="n">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="D32" t="n">
-        <v>28.89</v>
+        <v>30.74</v>
       </c>
     </row>
     <row r="33">
@@ -959,10 +959,10 @@
         <v>686</v>
       </c>
       <c r="C33" t="n">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D33" t="n">
-        <v>46.36</v>
+        <v>46.79</v>
       </c>
     </row>
     <row r="34">
@@ -991,10 +991,10 @@
         <v>163</v>
       </c>
       <c r="C35" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D35" t="n">
-        <v>77.3</v>
+        <v>77.91</v>
       </c>
     </row>
     <row r="36">
@@ -1007,10 +1007,10 @@
         <v>631</v>
       </c>
       <c r="C36" t="n">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D36" t="n">
-        <v>29.48</v>
+        <v>29.95</v>
       </c>
     </row>
     <row r="37">
@@ -1023,10 +1023,10 @@
         <v>385</v>
       </c>
       <c r="C37" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D37" t="n">
-        <v>27.79</v>
+        <v>28.31</v>
       </c>
     </row>
     <row r="38">
@@ -1055,10 +1055,10 @@
         <v>828</v>
       </c>
       <c r="C39" t="n">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D39" t="n">
-        <v>46.14</v>
+        <v>46.38</v>
       </c>
     </row>
     <row r="40">
@@ -1071,10 +1071,10 @@
         <v>300</v>
       </c>
       <c r="C40" t="n">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="D40" t="n">
-        <v>82.67</v>
+        <v>87.33</v>
       </c>
     </row>
     <row r="41">
@@ -1087,10 +1087,10 @@
         <v>406</v>
       </c>
       <c r="C41" t="n">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D41" t="n">
-        <v>51.23</v>
+        <v>52.71</v>
       </c>
     </row>
     <row r="42">
@@ -1103,10 +1103,10 @@
         <v>385</v>
       </c>
       <c r="C42" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D42" t="n">
-        <v>37.92</v>
+        <v>38.44</v>
       </c>
     </row>
     <row r="43">
@@ -1119,10 +1119,10 @@
         <v>335</v>
       </c>
       <c r="C43" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D43" t="n">
-        <v>8.359999999999999</v>
+        <v>8.66</v>
       </c>
     </row>
     <row r="44">
@@ -1135,10 +1135,10 @@
         <v>873</v>
       </c>
       <c r="C44" t="n">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="D44" t="n">
-        <v>47.65</v>
+        <v>48.34</v>
       </c>
     </row>
     <row r="45">
@@ -1167,10 +1167,10 @@
         <v>361</v>
       </c>
       <c r="C46" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="D46" t="n">
-        <v>28.81</v>
+        <v>32.69</v>
       </c>
     </row>
     <row r="47">
@@ -1183,10 +1183,10 @@
         <v>365</v>
       </c>
       <c r="C47" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D47" t="n">
-        <v>77.26000000000001</v>
+        <v>77.53</v>
       </c>
     </row>
     <row r="48">
@@ -1231,10 +1231,10 @@
         <v>1051</v>
       </c>
       <c r="C50" t="n">
-        <v>330</v>
+        <v>344</v>
       </c>
       <c r="D50" t="n">
-        <v>31.4</v>
+        <v>32.73</v>
       </c>
     </row>
     <row r="51">
@@ -1279,10 +1279,10 @@
         <v>516</v>
       </c>
       <c r="C53" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D53" t="n">
-        <v>17.25</v>
+        <v>17.64</v>
       </c>
     </row>
     <row r="54">
@@ -1311,10 +1311,10 @@
         <v>522</v>
       </c>
       <c r="C55" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D55" t="n">
-        <v>15.9</v>
+        <v>16.86</v>
       </c>
     </row>
     <row r="56">
@@ -1343,10 +1343,10 @@
         <v>347</v>
       </c>
       <c r="C57" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D57" t="n">
-        <v>47.84</v>
+        <v>48.41</v>
       </c>
     </row>
     <row r="58">
@@ -1359,10 +1359,10 @@
         <v>537</v>
       </c>
       <c r="C58" t="n">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="D58" t="n">
-        <v>39.29</v>
+        <v>41.53</v>
       </c>
     </row>
     <row r="59">
@@ -1391,10 +1391,10 @@
         <v>225</v>
       </c>
       <c r="C60" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D60" t="n">
-        <v>67.11</v>
+        <v>67.56</v>
       </c>
     </row>
     <row r="61">
@@ -1407,10 +1407,10 @@
         <v>742</v>
       </c>
       <c r="C61" t="n">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D61" t="n">
-        <v>34.91</v>
+        <v>35.31</v>
       </c>
     </row>
     <row r="62">
@@ -1423,10 +1423,10 @@
         <v>1181</v>
       </c>
       <c r="C62" t="n">
-        <v>231</v>
+        <v>248</v>
       </c>
       <c r="D62" t="n">
-        <v>19.56</v>
+        <v>21</v>
       </c>
     </row>
     <row r="63">
@@ -1455,10 +1455,10 @@
         <v>266</v>
       </c>
       <c r="C64" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D64" t="n">
-        <v>79.31999999999999</v>
+        <v>79.7</v>
       </c>
     </row>
     <row r="65">
@@ -1471,10 +1471,10 @@
         <v>452</v>
       </c>
       <c r="C65" t="n">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="D65" t="n">
-        <v>61.73</v>
+        <v>65.27</v>
       </c>
     </row>
     <row r="66">
@@ -1487,10 +1487,10 @@
         <v>262</v>
       </c>
       <c r="C66" t="n">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D66" t="n">
-        <v>72.14</v>
+        <v>77.09999999999999</v>
       </c>
     </row>
     <row r="67">
@@ -1503,10 +1503,10 @@
         <v>310</v>
       </c>
       <c r="C67" t="n">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="D67" t="n">
-        <v>20.97</v>
+        <v>34.19</v>
       </c>
     </row>
     <row r="68">
@@ -1535,10 +1535,10 @@
         <v>150</v>
       </c>
       <c r="C69" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D69" t="n">
-        <v>88.67</v>
+        <v>89.33</v>
       </c>
     </row>
     <row r="70">
@@ -1583,10 +1583,10 @@
         <v>468</v>
       </c>
       <c r="C72" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D72" t="n">
-        <v>68.16</v>
+        <v>68.38</v>
       </c>
     </row>
     <row r="73">
@@ -1599,10 +1599,10 @@
         <v>239</v>
       </c>
       <c r="C73" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D73" t="n">
-        <v>50.21</v>
+        <v>54.39</v>
       </c>
     </row>
     <row r="74">
@@ -1631,10 +1631,10 @@
         <v>435</v>
       </c>
       <c r="C75" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D75" t="n">
-        <v>88.51000000000001</v>
+        <v>88.73999999999999</v>
       </c>
     </row>
     <row r="76">
@@ -1647,10 +1647,10 @@
         <v>622</v>
       </c>
       <c r="C76" t="n">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D76" t="n">
-        <v>46.46</v>
+        <v>46.78</v>
       </c>
     </row>
     <row r="77">
@@ -1663,10 +1663,10 @@
         <v>33332</v>
       </c>
       <c r="C77" t="n">
-        <v>13386</v>
+        <v>13724</v>
       </c>
       <c r="D77" t="n">
-        <v>40.16</v>
+        <v>41.17</v>
       </c>
     </row>
   </sheetData>
@@ -1715,10 +1715,10 @@
         <v>150</v>
       </c>
       <c r="C2" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D2" t="n">
-        <v>88.67</v>
+        <v>89.33</v>
       </c>
     </row>
     <row r="3">
@@ -1731,10 +1731,10 @@
         <v>435</v>
       </c>
       <c r="C3" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D3" t="n">
-        <v>88.51000000000001</v>
+        <v>88.73999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1747,10 +1747,10 @@
         <v>300</v>
       </c>
       <c r="C4" t="n">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="D4" t="n">
-        <v>82.67</v>
+        <v>87.33</v>
       </c>
     </row>
     <row r="5">
@@ -1763,10 +1763,10 @@
         <v>266</v>
       </c>
       <c r="C5" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D5" t="n">
-        <v>79.31999999999999</v>
+        <v>79.7</v>
       </c>
     </row>
     <row r="6">
@@ -1779,10 +1779,10 @@
         <v>163</v>
       </c>
       <c r="C6" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D6" t="n">
-        <v>77.3</v>
+        <v>77.91</v>
       </c>
     </row>
     <row r="7">
@@ -1795,42 +1795,42 @@
         <v>365</v>
       </c>
       <c r="C7" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D7" t="n">
-        <v>77.26000000000001</v>
+        <v>77.53</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAHOBA</t>
+          <t>SAMBHAL (BHIM NAGAR)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>112</v>
+        <v>262</v>
       </c>
       <c r="C8" t="n">
-        <v>86</v>
+        <v>202</v>
       </c>
       <c r="D8" t="n">
-        <v>76.79000000000001</v>
+        <v>77.09999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAMBHAL (BHIM NAGAR)</t>
+          <t>MAHOBA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>262</v>
+        <v>112</v>
       </c>
       <c r="C9" t="n">
-        <v>189</v>
+        <v>86</v>
       </c>
       <c r="D9" t="n">
-        <v>72.14</v>
+        <v>76.79000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1843,10 +1843,10 @@
         <v>429</v>
       </c>
       <c r="C10" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D10" t="n">
-        <v>71.79000000000001</v>
+        <v>72.03</v>
       </c>
     </row>
     <row r="11">
@@ -1911,10 +1911,10 @@
         <v>335</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" t="n">
-        <v>8.359999999999999</v>
+        <v>8.66</v>
       </c>
     </row>
     <row r="3">
@@ -1927,10 +1927,10 @@
         <v>949</v>
       </c>
       <c r="C3" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="D3" t="n">
-        <v>9.59</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="4">
@@ -1943,10 +1943,10 @@
         <v>522</v>
       </c>
       <c r="C4" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D4" t="n">
-        <v>15.9</v>
+        <v>16.86</v>
       </c>
     </row>
     <row r="5">
@@ -1975,10 +1975,10 @@
         <v>516</v>
       </c>
       <c r="C6" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6" t="n">
-        <v>17.25</v>
+        <v>17.64</v>
       </c>
     </row>
     <row r="7">
@@ -2000,113 +2000,113 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PRAYAGRAJ</t>
+          <t>AZAMGARH</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1181</v>
+        <v>838</v>
       </c>
       <c r="C8" t="n">
-        <v>231</v>
+        <v>169</v>
       </c>
       <c r="D8" t="n">
-        <v>19.56</v>
+        <v>20.17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AZAMGARH</t>
+          <t>SHAHJAHANPUR</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>838</v>
+        <v>430</v>
       </c>
       <c r="C9" t="n">
-        <v>164</v>
+        <v>90</v>
       </c>
       <c r="D9" t="n">
-        <v>19.57</v>
+        <v>20.93</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SHAHJAHANPUR</t>
+          <t>PRAYAGRAJ</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>430</v>
+        <v>1181</v>
       </c>
       <c r="C10" t="n">
-        <v>90</v>
+        <v>248</v>
       </c>
       <c r="D10" t="n">
-        <v>20.93</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SANT KABIR NAGAR</t>
+          <t>ALIGARH</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>310</v>
+        <v>868</v>
       </c>
       <c r="C11" t="n">
-        <v>65</v>
+        <v>199</v>
       </c>
       <c r="D11" t="n">
-        <v>20.97</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALIGARH</t>
+          <t>ETAWAH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>868</v>
+        <v>313</v>
       </c>
       <c r="C12" t="n">
-        <v>199</v>
+        <v>73</v>
       </c>
       <c r="D12" t="n">
-        <v>22.93</v>
+        <v>23.32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ETAWAH</t>
+          <t>ETAH</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>313</v>
+        <v>561</v>
       </c>
       <c r="C13" t="n">
-        <v>73</v>
+        <v>131</v>
       </c>
       <c r="D13" t="n">
-        <v>23.32</v>
+        <v>23.35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ETAH</t>
+          <t>MATHURA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>561</v>
+        <v>640</v>
       </c>
       <c r="C14" t="n">
-        <v>131</v>
+        <v>169</v>
       </c>
       <c r="D14" t="n">
-        <v>23.35</v>
+        <v>26.41</v>
       </c>
     </row>
     <row r="15">
@@ -2119,154 +2119,154 @@
         <v>1077</v>
       </c>
       <c r="C15" t="n">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="D15" t="n">
-        <v>24.33</v>
+        <v>26.74</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MATHURA</t>
+          <t>HATHRAS</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>640</v>
+        <v>385</v>
       </c>
       <c r="C16" t="n">
-        <v>169</v>
+        <v>109</v>
       </c>
       <c r="D16" t="n">
-        <v>26.41</v>
+        <v>28.31</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HATHRAS</t>
+          <t>SIDDHARTHNAGAR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>385</v>
+        <v>246</v>
       </c>
       <c r="C17" t="n">
-        <v>107</v>
+        <v>73</v>
       </c>
       <c r="D17" t="n">
-        <v>27.79</v>
+        <v>29.67</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>KAUSHAMBI</t>
+          <t>HARDOI</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>361</v>
+        <v>631</v>
       </c>
       <c r="C18" t="n">
-        <v>104</v>
+        <v>189</v>
       </c>
       <c r="D18" t="n">
-        <v>28.81</v>
+        <v>29.95</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GONDA</t>
+          <t>BULANDSHAHR</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>540</v>
+        <v>524</v>
       </c>
       <c r="C19" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D19" t="n">
-        <v>28.89</v>
+        <v>30.34</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HARDOI</t>
+          <t>AURAIYA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>631</v>
+        <v>300</v>
       </c>
       <c r="C20" t="n">
-        <v>186</v>
+        <v>92</v>
       </c>
       <c r="D20" t="n">
-        <v>29.48</v>
+        <v>30.67</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SIDDHARTHNAGAR</t>
+          <t>GONDA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>246</v>
+        <v>540</v>
       </c>
       <c r="C21" t="n">
-        <v>73</v>
+        <v>166</v>
       </c>
       <c r="D21" t="n">
-        <v>29.67</v>
+        <v>30.74</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BULANDSHAHR</t>
+          <t>BAHRAICH</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>524</v>
+        <v>330</v>
       </c>
       <c r="C22" t="n">
-        <v>159</v>
+        <v>103</v>
       </c>
       <c r="D22" t="n">
-        <v>30.34</v>
+        <v>31.21</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AURAIYA</t>
+          <t>RAE BARELI</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>300</v>
+        <v>401</v>
       </c>
       <c r="C23" t="n">
-        <v>92</v>
+        <v>127</v>
       </c>
       <c r="D23" t="n">
-        <v>30.67</v>
+        <v>31.67</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BAHRAICH</t>
+          <t>KAUSHAMBI</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C24" t="n">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="D24" t="n">
-        <v>30.91</v>
+        <v>32.69</v>
       </c>
     </row>
     <row r="25">
@@ -2279,26 +2279,26 @@
         <v>1051</v>
       </c>
       <c r="C25" t="n">
-        <v>330</v>
+        <v>344</v>
       </c>
       <c r="D25" t="n">
-        <v>31.4</v>
+        <v>32.73</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RAE BARELI</t>
+          <t>SANT KABIR NAGAR</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>401</v>
+        <v>310</v>
       </c>
       <c r="C26" t="n">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="D26" t="n">
-        <v>31.67</v>
+        <v>34.19</v>
       </c>
     </row>
   </sheetData>
@@ -2344,7 +2344,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13386</v>
+        <v>13724</v>
       </c>
     </row>
     <row r="4">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40.16</v>
+        <v>41.17</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Update data files from local development
</commit_message>
<xml_diff>
--- a/Eco-Club-Complete_Summary.xlsx
+++ b/Eco-Club-Complete_Summary.xlsx
@@ -463,10 +463,10 @@
         <v>1077</v>
       </c>
       <c r="C2" t="n">
-        <v>288</v>
+        <v>319</v>
       </c>
       <c r="D2" t="n">
-        <v>26.74</v>
+        <v>29.62</v>
       </c>
     </row>
     <row r="3">
@@ -495,10 +495,10 @@
         <v>429</v>
       </c>
       <c r="C4" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D4" t="n">
-        <v>72.03</v>
+        <v>72.73</v>
       </c>
     </row>
     <row r="5">
@@ -511,10 +511,10 @@
         <v>274</v>
       </c>
       <c r="C5" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D5" t="n">
-        <v>52.55</v>
+        <v>52.92</v>
       </c>
     </row>
     <row r="6">
@@ -543,10 +543,10 @@
         <v>838</v>
       </c>
       <c r="C7" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D7" t="n">
-        <v>20.17</v>
+        <v>20.41</v>
       </c>
     </row>
     <row r="8">
@@ -559,10 +559,10 @@
         <v>218</v>
       </c>
       <c r="C8" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D8" t="n">
-        <v>42.66</v>
+        <v>43.12</v>
       </c>
     </row>
     <row r="9">
@@ -575,10 +575,10 @@
         <v>330</v>
       </c>
       <c r="C9" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D9" t="n">
-        <v>31.21</v>
+        <v>32.12</v>
       </c>
     </row>
     <row r="10">
@@ -591,10 +591,10 @@
         <v>625</v>
       </c>
       <c r="C10" t="n">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D10" t="n">
-        <v>37.28</v>
+        <v>37.76</v>
       </c>
     </row>
     <row r="11">
@@ -671,10 +671,10 @@
         <v>442</v>
       </c>
       <c r="C15" t="n">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D15" t="n">
-        <v>40.72</v>
+        <v>42.08</v>
       </c>
     </row>
     <row r="16">
@@ -687,10 +687,10 @@
         <v>231</v>
       </c>
       <c r="C16" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D16" t="n">
-        <v>61.9</v>
+        <v>62.34</v>
       </c>
     </row>
     <row r="17">
@@ -703,10 +703,10 @@
         <v>528</v>
       </c>
       <c r="C17" t="n">
-        <v>290</v>
+        <v>313</v>
       </c>
       <c r="D17" t="n">
-        <v>54.92</v>
+        <v>59.28</v>
       </c>
     </row>
     <row r="18">
@@ -719,10 +719,10 @@
         <v>324</v>
       </c>
       <c r="C18" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" t="n">
-        <v>34.26</v>
+        <v>34.57</v>
       </c>
     </row>
     <row r="19">
@@ -767,10 +767,10 @@
         <v>134</v>
       </c>
       <c r="C21" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D21" t="n">
-        <v>64.18000000000001</v>
+        <v>64.93000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -799,10 +799,10 @@
         <v>561</v>
       </c>
       <c r="C23" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D23" t="n">
-        <v>23.35</v>
+        <v>23.53</v>
       </c>
     </row>
     <row r="24">
@@ -847,10 +847,10 @@
         <v>323</v>
       </c>
       <c r="C26" t="n">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="D26" t="n">
-        <v>49.85</v>
+        <v>53.25</v>
       </c>
     </row>
     <row r="27">
@@ -863,10 +863,10 @@
         <v>463</v>
       </c>
       <c r="C27" t="n">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="D27" t="n">
-        <v>58.1</v>
+        <v>61.12</v>
       </c>
     </row>
     <row r="28">
@@ -879,10 +879,10 @@
         <v>614</v>
       </c>
       <c r="C28" t="n">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D28" t="n">
-        <v>46.91</v>
+        <v>47.39</v>
       </c>
     </row>
     <row r="29">
@@ -927,10 +927,10 @@
         <v>949</v>
       </c>
       <c r="C31" t="n">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D31" t="n">
-        <v>11.49</v>
+        <v>12.22</v>
       </c>
     </row>
     <row r="32">
@@ -943,10 +943,10 @@
         <v>540</v>
       </c>
       <c r="C32" t="n">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D32" t="n">
-        <v>30.74</v>
+        <v>32.41</v>
       </c>
     </row>
     <row r="33">
@@ -959,10 +959,10 @@
         <v>686</v>
       </c>
       <c r="C33" t="n">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D33" t="n">
-        <v>46.79</v>
+        <v>47.08</v>
       </c>
     </row>
     <row r="34">
@@ -1007,10 +1007,10 @@
         <v>631</v>
       </c>
       <c r="C36" t="n">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D36" t="n">
-        <v>29.95</v>
+        <v>30.27</v>
       </c>
     </row>
     <row r="37">
@@ -1023,10 +1023,10 @@
         <v>385</v>
       </c>
       <c r="C37" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D37" t="n">
-        <v>28.31</v>
+        <v>28.83</v>
       </c>
     </row>
     <row r="38">
@@ -1055,10 +1055,10 @@
         <v>828</v>
       </c>
       <c r="C39" t="n">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="D39" t="n">
-        <v>46.38</v>
+        <v>46.98</v>
       </c>
     </row>
     <row r="40">
@@ -1071,10 +1071,10 @@
         <v>300</v>
       </c>
       <c r="C40" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D40" t="n">
-        <v>87.33</v>
+        <v>88.67</v>
       </c>
     </row>
     <row r="41">
@@ -1087,10 +1087,10 @@
         <v>406</v>
       </c>
       <c r="C41" t="n">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D41" t="n">
-        <v>52.71</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="42">
@@ -1135,10 +1135,10 @@
         <v>873</v>
       </c>
       <c r="C44" t="n">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="D44" t="n">
-        <v>48.34</v>
+        <v>48.8</v>
       </c>
     </row>
     <row r="45">
@@ -1167,10 +1167,10 @@
         <v>361</v>
       </c>
       <c r="C46" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D46" t="n">
-        <v>32.69</v>
+        <v>32.96</v>
       </c>
     </row>
     <row r="47">
@@ -1183,10 +1183,10 @@
         <v>365</v>
       </c>
       <c r="C47" t="n">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D47" t="n">
-        <v>77.53</v>
+        <v>78.63</v>
       </c>
     </row>
     <row r="48">
@@ -1199,10 +1199,10 @@
         <v>413</v>
       </c>
       <c r="C48" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D48" t="n">
-        <v>17.19</v>
+        <v>17.92</v>
       </c>
     </row>
     <row r="49">
@@ -1231,10 +1231,10 @@
         <v>1051</v>
       </c>
       <c r="C50" t="n">
-        <v>344</v>
+        <v>372</v>
       </c>
       <c r="D50" t="n">
-        <v>32.73</v>
+        <v>35.39</v>
       </c>
     </row>
     <row r="51">
@@ -1263,10 +1263,10 @@
         <v>112</v>
       </c>
       <c r="C52" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D52" t="n">
-        <v>76.79000000000001</v>
+        <v>77.68000000000001</v>
       </c>
     </row>
     <row r="53">
@@ -1279,10 +1279,10 @@
         <v>516</v>
       </c>
       <c r="C53" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D53" t="n">
-        <v>17.64</v>
+        <v>18.22</v>
       </c>
     </row>
     <row r="54">
@@ -1295,10 +1295,10 @@
         <v>640</v>
       </c>
       <c r="C54" t="n">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D54" t="n">
-        <v>26.41</v>
+        <v>27.19</v>
       </c>
     </row>
     <row r="55">
@@ -1311,10 +1311,10 @@
         <v>522</v>
       </c>
       <c r="C55" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D55" t="n">
-        <v>16.86</v>
+        <v>17.82</v>
       </c>
     </row>
     <row r="56">
@@ -1343,10 +1343,10 @@
         <v>347</v>
       </c>
       <c r="C57" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D57" t="n">
-        <v>48.41</v>
+        <v>48.7</v>
       </c>
     </row>
     <row r="58">
@@ -1359,10 +1359,10 @@
         <v>537</v>
       </c>
       <c r="C58" t="n">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="D58" t="n">
-        <v>41.53</v>
+        <v>43.95</v>
       </c>
     </row>
     <row r="59">
@@ -1375,10 +1375,10 @@
         <v>388</v>
       </c>
       <c r="C59" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D59" t="n">
-        <v>52.84</v>
+        <v>53.09</v>
       </c>
     </row>
     <row r="60">
@@ -1407,10 +1407,10 @@
         <v>742</v>
       </c>
       <c r="C61" t="n">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D61" t="n">
-        <v>35.31</v>
+        <v>35.58</v>
       </c>
     </row>
     <row r="62">
@@ -1423,10 +1423,10 @@
         <v>1181</v>
       </c>
       <c r="C62" t="n">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="D62" t="n">
-        <v>21</v>
+        <v>21.42</v>
       </c>
     </row>
     <row r="63">
@@ -1471,10 +1471,10 @@
         <v>452</v>
       </c>
       <c r="C65" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D65" t="n">
-        <v>65.27</v>
+        <v>65.48999999999999</v>
       </c>
     </row>
     <row r="66">
@@ -1503,10 +1503,10 @@
         <v>310</v>
       </c>
       <c r="C67" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D67" t="n">
-        <v>34.19</v>
+        <v>35.81</v>
       </c>
     </row>
     <row r="68">
@@ -1519,10 +1519,10 @@
         <v>430</v>
       </c>
       <c r="C68" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D68" t="n">
-        <v>20.93</v>
+        <v>21.16</v>
       </c>
     </row>
     <row r="69">
@@ -1535,10 +1535,10 @@
         <v>150</v>
       </c>
       <c r="C69" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D69" t="n">
-        <v>89.33</v>
+        <v>90.67</v>
       </c>
     </row>
     <row r="70">
@@ -1599,10 +1599,10 @@
         <v>239</v>
       </c>
       <c r="C73" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D73" t="n">
-        <v>54.39</v>
+        <v>55.23</v>
       </c>
     </row>
     <row r="74">
@@ -1631,10 +1631,10 @@
         <v>435</v>
       </c>
       <c r="C75" t="n">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D75" t="n">
-        <v>88.73999999999999</v>
+        <v>89.66</v>
       </c>
     </row>
     <row r="76">
@@ -1647,10 +1647,10 @@
         <v>622</v>
       </c>
       <c r="C76" t="n">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="D76" t="n">
-        <v>46.78</v>
+        <v>48.07</v>
       </c>
     </row>
     <row r="77">
@@ -1663,10 +1663,10 @@
         <v>33332</v>
       </c>
       <c r="C77" t="n">
-        <v>13724</v>
+        <v>13961</v>
       </c>
       <c r="D77" t="n">
-        <v>41.17</v>
+        <v>41.88</v>
       </c>
     </row>
   </sheetData>
@@ -1715,10 +1715,10 @@
         <v>150</v>
       </c>
       <c r="C2" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D2" t="n">
-        <v>89.33</v>
+        <v>90.67</v>
       </c>
     </row>
     <row r="3">
@@ -1731,10 +1731,10 @@
         <v>435</v>
       </c>
       <c r="C3" t="n">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D3" t="n">
-        <v>88.73999999999999</v>
+        <v>89.66</v>
       </c>
     </row>
     <row r="4">
@@ -1747,10 +1747,10 @@
         <v>300</v>
       </c>
       <c r="C4" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D4" t="n">
-        <v>87.33</v>
+        <v>88.67</v>
       </c>
     </row>
     <row r="5">
@@ -1772,65 +1772,65 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HAPUR (PANCHSHEEL NAGAR)</t>
+          <t>KHERI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>163</v>
+        <v>365</v>
       </c>
       <c r="C6" t="n">
-        <v>127</v>
+        <v>287</v>
       </c>
       <c r="D6" t="n">
-        <v>77.91</v>
+        <v>78.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KHERI</t>
+          <t>HAPUR (PANCHSHEEL NAGAR)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>365</v>
+        <v>163</v>
       </c>
       <c r="C7" t="n">
-        <v>283</v>
+        <v>127</v>
       </c>
       <c r="D7" t="n">
-        <v>77.53</v>
+        <v>77.91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAMBHAL (BHIM NAGAR)</t>
+          <t>MAHOBA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>262</v>
+        <v>112</v>
       </c>
       <c r="C8" t="n">
-        <v>202</v>
+        <v>87</v>
       </c>
       <c r="D8" t="n">
-        <v>77.09999999999999</v>
+        <v>77.68000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MAHOBA</t>
+          <t>SAMBHAL (BHIM NAGAR)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>112</v>
+        <v>262</v>
       </c>
       <c r="C9" t="n">
-        <v>86</v>
+        <v>202</v>
       </c>
       <c r="D9" t="n">
-        <v>76.79000000000001</v>
+        <v>77.09999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1843,10 +1843,10 @@
         <v>429</v>
       </c>
       <c r="C10" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D10" t="n">
-        <v>72.03</v>
+        <v>72.73</v>
       </c>
     </row>
     <row r="11">
@@ -1927,10 +1927,10 @@
         <v>949</v>
       </c>
       <c r="C3" t="n">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D3" t="n">
-        <v>11.49</v>
+        <v>12.22</v>
       </c>
     </row>
     <row r="4">
@@ -1943,10 +1943,10 @@
         <v>522</v>
       </c>
       <c r="C4" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D4" t="n">
-        <v>16.86</v>
+        <v>17.82</v>
       </c>
     </row>
     <row r="5">
@@ -1959,10 +1959,10 @@
         <v>413</v>
       </c>
       <c r="C5" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D5" t="n">
-        <v>17.19</v>
+        <v>17.92</v>
       </c>
     </row>
     <row r="6">
@@ -1975,10 +1975,10 @@
         <v>516</v>
       </c>
       <c r="C6" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D6" t="n">
-        <v>17.64</v>
+        <v>18.22</v>
       </c>
     </row>
     <row r="7">
@@ -2007,10 +2007,10 @@
         <v>838</v>
       </c>
       <c r="C8" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D8" t="n">
-        <v>20.17</v>
+        <v>20.41</v>
       </c>
     </row>
     <row r="9">
@@ -2023,10 +2023,10 @@
         <v>430</v>
       </c>
       <c r="C9" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D9" t="n">
-        <v>20.93</v>
+        <v>21.16</v>
       </c>
     </row>
     <row r="10">
@@ -2039,10 +2039,10 @@
         <v>1181</v>
       </c>
       <c r="C10" t="n">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>21.42</v>
       </c>
     </row>
     <row r="11">
@@ -2087,10 +2087,10 @@
         <v>561</v>
       </c>
       <c r="C13" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D13" t="n">
-        <v>23.35</v>
+        <v>23.53</v>
       </c>
     </row>
     <row r="14">
@@ -2103,42 +2103,42 @@
         <v>640</v>
       </c>
       <c r="C14" t="n">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D14" t="n">
-        <v>26.41</v>
+        <v>27.19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AGRA</t>
+          <t>HATHRAS</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1077</v>
+        <v>385</v>
       </c>
       <c r="C15" t="n">
-        <v>288</v>
+        <v>111</v>
       </c>
       <c r="D15" t="n">
-        <v>26.74</v>
+        <v>28.83</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HATHRAS</t>
+          <t>AGRA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>385</v>
+        <v>1077</v>
       </c>
       <c r="C16" t="n">
-        <v>109</v>
+        <v>319</v>
       </c>
       <c r="D16" t="n">
-        <v>28.31</v>
+        <v>29.62</v>
       </c>
     </row>
     <row r="17">
@@ -2167,10 +2167,10 @@
         <v>631</v>
       </c>
       <c r="C18" t="n">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D18" t="n">
-        <v>29.95</v>
+        <v>30.27</v>
       </c>
     </row>
     <row r="19">
@@ -2208,17 +2208,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GONDA</t>
+          <t>RAE BARELI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>540</v>
+        <v>401</v>
       </c>
       <c r="C21" t="n">
-        <v>166</v>
+        <v>127</v>
       </c>
       <c r="D21" t="n">
-        <v>30.74</v>
+        <v>31.67</v>
       </c>
     </row>
     <row r="22">
@@ -2231,26 +2231,26 @@
         <v>330</v>
       </c>
       <c r="C22" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D22" t="n">
-        <v>31.21</v>
+        <v>32.12</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RAE BARELI</t>
+          <t>GONDA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>401</v>
+        <v>540</v>
       </c>
       <c r="C23" t="n">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="D23" t="n">
-        <v>31.67</v>
+        <v>32.41</v>
       </c>
     </row>
     <row r="24">
@@ -2263,42 +2263,42 @@
         <v>361</v>
       </c>
       <c r="C24" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D24" t="n">
-        <v>32.69</v>
+        <v>32.96</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LUCKNOW</t>
+          <t>BUDAUN</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1051</v>
+        <v>324</v>
       </c>
       <c r="C25" t="n">
-        <v>344</v>
+        <v>112</v>
       </c>
       <c r="D25" t="n">
-        <v>32.73</v>
+        <v>34.57</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SANT KABIR NAGAR</t>
+          <t>LUCKNOW</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>310</v>
+        <v>1051</v>
       </c>
       <c r="C26" t="n">
-        <v>106</v>
+        <v>372</v>
       </c>
       <c r="D26" t="n">
-        <v>34.19</v>
+        <v>35.39</v>
       </c>
     </row>
   </sheetData>
@@ -2344,7 +2344,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13724</v>
+        <v>13961</v>
       </c>
     </row>
     <row r="4">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41.17</v>
+        <v>41.88</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Updated Eco Club data and added comprehensive reports - Jan 9, 2026
</commit_message>
<xml_diff>
--- a/Eco-Club-Complete_Summary.xlsx
+++ b/Eco-Club-Complete_Summary.xlsx
@@ -463,10 +463,10 @@
         <v>1077</v>
       </c>
       <c r="C2" t="n">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="D2" t="n">
-        <v>29.62</v>
+        <v>30.27</v>
       </c>
     </row>
     <row r="3">
@@ -495,10 +495,10 @@
         <v>429</v>
       </c>
       <c r="C4" t="n">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D4" t="n">
-        <v>72.73</v>
+        <v>73.89</v>
       </c>
     </row>
     <row r="5">
@@ -543,10 +543,10 @@
         <v>838</v>
       </c>
       <c r="C7" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D7" t="n">
-        <v>20.41</v>
+        <v>20.76</v>
       </c>
     </row>
     <row r="8">
@@ -559,10 +559,10 @@
         <v>218</v>
       </c>
       <c r="C8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D8" t="n">
-        <v>43.12</v>
+        <v>43.58</v>
       </c>
     </row>
     <row r="9">
@@ -591,10 +591,10 @@
         <v>625</v>
       </c>
       <c r="C10" t="n">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D10" t="n">
-        <v>37.76</v>
+        <v>38.08</v>
       </c>
     </row>
     <row r="11">
@@ -671,10 +671,10 @@
         <v>442</v>
       </c>
       <c r="C15" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D15" t="n">
-        <v>42.08</v>
+        <v>42.53</v>
       </c>
     </row>
     <row r="16">
@@ -687,10 +687,10 @@
         <v>231</v>
       </c>
       <c r="C16" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D16" t="n">
-        <v>62.34</v>
+        <v>63.2</v>
       </c>
     </row>
     <row r="17">
@@ -703,10 +703,10 @@
         <v>528</v>
       </c>
       <c r="C17" t="n">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="D17" t="n">
-        <v>59.28</v>
+        <v>61.36</v>
       </c>
     </row>
     <row r="18">
@@ -719,10 +719,10 @@
         <v>324</v>
       </c>
       <c r="C18" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D18" t="n">
-        <v>34.57</v>
+        <v>34.88</v>
       </c>
     </row>
     <row r="19">
@@ -735,10 +735,10 @@
         <v>524</v>
       </c>
       <c r="C19" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D19" t="n">
-        <v>30.34</v>
+        <v>30.53</v>
       </c>
     </row>
     <row r="20">
@@ -751,10 +751,10 @@
         <v>290</v>
       </c>
       <c r="C20" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D20" t="n">
-        <v>70</v>
+        <v>70.69</v>
       </c>
     </row>
     <row r="21">
@@ -767,10 +767,10 @@
         <v>134</v>
       </c>
       <c r="C21" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D21" t="n">
-        <v>64.93000000000001</v>
+        <v>65.67</v>
       </c>
     </row>
     <row r="22">
@@ -799,10 +799,10 @@
         <v>561</v>
       </c>
       <c r="C23" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D23" t="n">
-        <v>23.53</v>
+        <v>23.71</v>
       </c>
     </row>
     <row r="24">
@@ -815,10 +815,10 @@
         <v>313</v>
       </c>
       <c r="C24" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D24" t="n">
-        <v>23.32</v>
+        <v>23.64</v>
       </c>
     </row>
     <row r="25">
@@ -847,10 +847,10 @@
         <v>323</v>
       </c>
       <c r="C26" t="n">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="D26" t="n">
-        <v>53.25</v>
+        <v>55.11</v>
       </c>
     </row>
     <row r="27">
@@ -863,10 +863,10 @@
         <v>463</v>
       </c>
       <c r="C27" t="n">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="D27" t="n">
-        <v>61.12</v>
+        <v>62.85</v>
       </c>
     </row>
     <row r="28">
@@ -879,10 +879,10 @@
         <v>614</v>
       </c>
       <c r="C28" t="n">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="D28" t="n">
-        <v>47.39</v>
+        <v>48.7</v>
       </c>
     </row>
     <row r="29">
@@ -895,10 +895,10 @@
         <v>389</v>
       </c>
       <c r="C29" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D29" t="n">
-        <v>41.65</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="30">
@@ -943,10 +943,10 @@
         <v>540</v>
       </c>
       <c r="C32" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D32" t="n">
-        <v>32.41</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="33">
@@ -991,10 +991,10 @@
         <v>163</v>
       </c>
       <c r="C35" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D35" t="n">
-        <v>77.91</v>
+        <v>78.53</v>
       </c>
     </row>
     <row r="36">
@@ -1007,10 +1007,10 @@
         <v>631</v>
       </c>
       <c r="C36" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D36" t="n">
-        <v>30.27</v>
+        <v>30.59</v>
       </c>
     </row>
     <row r="37">
@@ -1023,10 +1023,10 @@
         <v>385</v>
       </c>
       <c r="C37" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D37" t="n">
-        <v>28.83</v>
+        <v>29.09</v>
       </c>
     </row>
     <row r="38">
@@ -1071,10 +1071,10 @@
         <v>300</v>
       </c>
       <c r="C40" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D40" t="n">
-        <v>88.67</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41">
@@ -1087,10 +1087,10 @@
         <v>406</v>
       </c>
       <c r="C41" t="n">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D41" t="n">
-        <v>53.2</v>
+        <v>53.69</v>
       </c>
     </row>
     <row r="42">
@@ -1135,10 +1135,10 @@
         <v>873</v>
       </c>
       <c r="C44" t="n">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D44" t="n">
-        <v>48.8</v>
+        <v>48.91</v>
       </c>
     </row>
     <row r="45">
@@ -1231,10 +1231,10 @@
         <v>1051</v>
       </c>
       <c r="C50" t="n">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="D50" t="n">
-        <v>35.39</v>
+        <v>36.92</v>
       </c>
     </row>
     <row r="51">
@@ -1263,10 +1263,10 @@
         <v>112</v>
       </c>
       <c r="C52" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D52" t="n">
-        <v>77.68000000000001</v>
+        <v>78.56999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -1295,10 +1295,10 @@
         <v>640</v>
       </c>
       <c r="C54" t="n">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="D54" t="n">
-        <v>27.19</v>
+        <v>30.47</v>
       </c>
     </row>
     <row r="55">
@@ -1311,10 +1311,10 @@
         <v>522</v>
       </c>
       <c r="C55" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D55" t="n">
-        <v>17.82</v>
+        <v>18.39</v>
       </c>
     </row>
     <row r="56">
@@ -1359,10 +1359,10 @@
         <v>537</v>
       </c>
       <c r="C58" t="n">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="D58" t="n">
-        <v>43.95</v>
+        <v>46.93</v>
       </c>
     </row>
     <row r="59">
@@ -1407,10 +1407,10 @@
         <v>742</v>
       </c>
       <c r="C61" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D61" t="n">
-        <v>35.58</v>
+        <v>35.71</v>
       </c>
     </row>
     <row r="62">
@@ -1423,10 +1423,10 @@
         <v>1181</v>
       </c>
       <c r="C62" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D62" t="n">
-        <v>21.42</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="63">
@@ -1519,10 +1519,10 @@
         <v>430</v>
       </c>
       <c r="C68" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D68" t="n">
-        <v>21.16</v>
+        <v>21.63</v>
       </c>
     </row>
     <row r="69">
@@ -1567,10 +1567,10 @@
         <v>246</v>
       </c>
       <c r="C71" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D71" t="n">
-        <v>29.67</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="72">
@@ -1599,10 +1599,10 @@
         <v>239</v>
       </c>
       <c r="C73" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D73" t="n">
-        <v>55.23</v>
+        <v>56.07</v>
       </c>
     </row>
     <row r="74">
@@ -1647,10 +1647,10 @@
         <v>622</v>
       </c>
       <c r="C76" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D76" t="n">
-        <v>48.07</v>
+        <v>48.23</v>
       </c>
     </row>
     <row r="77">
@@ -1663,10 +1663,10 @@
         <v>33332</v>
       </c>
       <c r="C77" t="n">
-        <v>13961</v>
+        <v>14111</v>
       </c>
       <c r="D77" t="n">
-        <v>41.88</v>
+        <v>42.33</v>
       </c>
     </row>
   </sheetData>
@@ -1747,10 +1747,10 @@
         <v>300</v>
       </c>
       <c r="C4" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D4" t="n">
-        <v>88.67</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5">
@@ -1788,33 +1788,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HAPUR (PANCHSHEEL NAGAR)</t>
+          <t>MAHOBA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>163</v>
+        <v>112</v>
       </c>
       <c r="C7" t="n">
-        <v>127</v>
+        <v>88</v>
       </c>
       <c r="D7" t="n">
-        <v>77.91</v>
+        <v>78.56999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAHOBA</t>
+          <t>HAPUR (PANCHSHEEL NAGAR)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>112</v>
+        <v>163</v>
       </c>
       <c r="C8" t="n">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="D8" t="n">
-        <v>77.68000000000001</v>
+        <v>78.53</v>
       </c>
     </row>
     <row r="9">
@@ -1843,10 +1843,10 @@
         <v>429</v>
       </c>
       <c r="C10" t="n">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D10" t="n">
-        <v>72.73</v>
+        <v>73.89</v>
       </c>
     </row>
     <row r="11">
@@ -1859,10 +1859,10 @@
         <v>290</v>
       </c>
       <c r="C11" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D11" t="n">
-        <v>70</v>
+        <v>70.69</v>
       </c>
     </row>
   </sheetData>
@@ -1936,49 +1936,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MAU</t>
+          <t>KUSHINAGAR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>522</v>
+        <v>413</v>
       </c>
       <c r="C4" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="D4" t="n">
-        <v>17.82</v>
+        <v>17.92</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KUSHINAGAR</t>
+          <t>MAINPURI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>413</v>
+        <v>516</v>
       </c>
       <c r="C5" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="D5" t="n">
-        <v>17.92</v>
+        <v>18.22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAINPURI</t>
+          <t>MAU</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="C6" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6" t="n">
-        <v>18.22</v>
+        <v>18.39</v>
       </c>
     </row>
     <row r="7">
@@ -2007,42 +2007,42 @@
         <v>838</v>
       </c>
       <c r="C8" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D8" t="n">
-        <v>20.41</v>
+        <v>20.76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SHAHJAHANPUR</t>
+          <t>PRAYAGRAJ</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>430</v>
+        <v>1181</v>
       </c>
       <c r="C9" t="n">
-        <v>91</v>
+        <v>255</v>
       </c>
       <c r="D9" t="n">
-        <v>21.16</v>
+        <v>21.59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PRAYAGRAJ</t>
+          <t>SHAHJAHANPUR</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1181</v>
+        <v>430</v>
       </c>
       <c r="C10" t="n">
-        <v>253</v>
+        <v>93</v>
       </c>
       <c r="D10" t="n">
-        <v>21.42</v>
+        <v>21.63</v>
       </c>
     </row>
     <row r="11">
@@ -2071,10 +2071,10 @@
         <v>313</v>
       </c>
       <c r="C12" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D12" t="n">
-        <v>23.32</v>
+        <v>23.64</v>
       </c>
     </row>
     <row r="13">
@@ -2087,74 +2087,74 @@
         <v>561</v>
       </c>
       <c r="C13" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D13" t="n">
-        <v>23.53</v>
+        <v>23.71</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MATHURA</t>
+          <t>HATHRAS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>640</v>
+        <v>385</v>
       </c>
       <c r="C14" t="n">
-        <v>174</v>
+        <v>112</v>
       </c>
       <c r="D14" t="n">
-        <v>27.19</v>
+        <v>29.09</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HATHRAS</t>
+          <t>AGRA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>385</v>
+        <v>1077</v>
       </c>
       <c r="C15" t="n">
-        <v>111</v>
+        <v>326</v>
       </c>
       <c r="D15" t="n">
-        <v>28.83</v>
+        <v>30.27</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGRA</t>
+          <t>MATHURA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1077</v>
+        <v>640</v>
       </c>
       <c r="C16" t="n">
-        <v>319</v>
+        <v>195</v>
       </c>
       <c r="D16" t="n">
-        <v>29.62</v>
+        <v>30.47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SIDDHARTHNAGAR</t>
+          <t>BULANDSHAHR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>246</v>
+        <v>524</v>
       </c>
       <c r="C17" t="n">
-        <v>73</v>
+        <v>160</v>
       </c>
       <c r="D17" t="n">
-        <v>29.67</v>
+        <v>30.53</v>
       </c>
     </row>
     <row r="18">
@@ -2167,74 +2167,74 @@
         <v>631</v>
       </c>
       <c r="C18" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D18" t="n">
-        <v>30.27</v>
+        <v>30.59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BULANDSHAHR</t>
+          <t>AURAIYA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>524</v>
+        <v>300</v>
       </c>
       <c r="C19" t="n">
-        <v>159</v>
+        <v>92</v>
       </c>
       <c r="D19" t="n">
-        <v>30.34</v>
+        <v>30.67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AURAIYA</t>
+          <t>RAE BARELI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>300</v>
+        <v>401</v>
       </c>
       <c r="C20" t="n">
-        <v>92</v>
+        <v>127</v>
       </c>
       <c r="D20" t="n">
-        <v>30.67</v>
+        <v>31.67</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RAE BARELI</t>
+          <t>BAHRAICH</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>401</v>
+        <v>330</v>
       </c>
       <c r="C21" t="n">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="D21" t="n">
-        <v>31.67</v>
+        <v>32.12</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAHRAICH</t>
+          <t>KAUSHAMBI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C22" t="n">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="D22" t="n">
-        <v>32.12</v>
+        <v>32.96</v>
       </c>
     </row>
     <row r="23">
@@ -2247,26 +2247,26 @@
         <v>540</v>
       </c>
       <c r="C23" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D23" t="n">
-        <v>32.41</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KAUSHAMBI</t>
+          <t>SIDDHARTHNAGAR</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>361</v>
+        <v>246</v>
       </c>
       <c r="C24" t="n">
-        <v>119</v>
+        <v>82</v>
       </c>
       <c r="D24" t="n">
-        <v>32.96</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="25">
@@ -2279,26 +2279,26 @@
         <v>324</v>
       </c>
       <c r="C25" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D25" t="n">
-        <v>34.57</v>
+        <v>34.88</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LUCKNOW</t>
+          <t>PRATAPGARH</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1051</v>
+        <v>742</v>
       </c>
       <c r="C26" t="n">
-        <v>372</v>
+        <v>265</v>
       </c>
       <c r="D26" t="n">
-        <v>35.39</v>
+        <v>35.71</v>
       </c>
     </row>
   </sheetData>
@@ -2344,7 +2344,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13961</v>
+        <v>14111</v>
       </c>
     </row>
     <row r="4">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41.88</v>
+        <v>42.33</v>
       </c>
     </row>
     <row r="5">

</xml_diff>